<commit_message>
used iferror, istext, isnumber
</commit_message>
<xml_diff>
--- a/Create from selection and Dates - Stu.xlsx
+++ b/Create from selection and Dates - Stu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Documents\Downloads\class\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C65A3ABD-ABA2-4908-84F0-AD0A46132BF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27FAC033-E499-4BCA-9F86-7E5BFF5776BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Create from selection" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="230">
   <si>
     <t>Month</t>
   </si>
@@ -714,6 +714,27 @@
   </si>
   <si>
     <t>Retirement Month</t>
+  </si>
+  <si>
+    <t>Total Delivery Days</t>
+  </si>
+  <si>
+    <t>Delivery Month</t>
+  </si>
+  <si>
+    <t>Weekday</t>
+  </si>
+  <si>
+    <t>Birth Month</t>
+  </si>
+  <si>
+    <t>Birth Weekday</t>
+  </si>
+  <si>
+    <t>Birth day</t>
+  </si>
+  <si>
+    <t>Next Birthday Year</t>
   </si>
 </sst>
 </file>
@@ -785,7 +806,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -828,11 +849,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -898,6 +932,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1569,7 +1609,7 @@
       </c>
       <c r="G3" s="9">
         <f ca="1">NOW()</f>
-        <v>46289.482888425926</v>
+        <v>46289.799810532408</v>
       </c>
       <c r="H3" s="10">
         <v>46227.947916666664</v>
@@ -1655,7 +1695,7 @@
       </c>
       <c r="L5" s="9">
         <f ca="1">NOW()</f>
-        <v>46289.482888425926</v>
+        <v>46289.799810532408</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="29">
@@ -2797,23 +2837,25 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6F2DCC1-8ED5-42B7-B182-90C462B3926A}">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
+    <col min="4" max="4" width="10.08984375" customWidth="1"/>
+    <col min="7" max="7" width="10.6328125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="31">
+    <row r="1" spans="1:7" ht="31">
       <c r="A1" s="13" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="23.5">
+    <row r="3" spans="1:7" ht="23.5">
       <c r="A3" s="12" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="29">
+    <row r="5" spans="1:7" ht="43.5">
       <c r="A5" s="3" t="s">
         <v>123</v>
       </c>
@@ -2823,8 +2865,20 @@
       <c r="C5" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="D5" s="28" t="s">
+        <v>223</v>
+      </c>
+      <c r="E5" s="28" t="s">
+        <v>215</v>
+      </c>
+      <c r="F5" s="28" t="s">
+        <v>224</v>
+      </c>
+      <c r="G5" s="28" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" s="2" t="s">
         <v>125</v>
       </c>
@@ -2834,8 +2888,24 @@
       <c r="C6" s="7">
         <v>46224</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
+      <c r="D6" s="19">
+        <f>DATEDIF('Exercise-2'!B6,'Exercise-2'!C6,"YD")</f>
+        <v>6</v>
+      </c>
+      <c r="E6" s="19">
+        <f>NETWORKDAYS(B6,C6)</f>
+        <v>5</v>
+      </c>
+      <c r="F6" s="19" t="str">
+        <f>TEXT(C6,"mmmm")</f>
+        <v>July</v>
+      </c>
+      <c r="G6" s="19" t="str">
+        <f>TEXT(C6,"dddd")</f>
+        <v>Tuesday</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7" s="2" t="s">
         <v>126</v>
       </c>
@@ -2845,8 +2915,24 @@
       <c r="C7" s="7">
         <v>46227</v>
       </c>
-    </row>
-    <row r="8" spans="1:3">
+      <c r="D7" s="19">
+        <f>DATEDIF('Exercise-2'!B7,'Exercise-2'!C7,"YD")</f>
+        <v>8</v>
+      </c>
+      <c r="E7" s="19">
+        <f t="shared" ref="E7:E10" si="0">NETWORKDAYS(B7,C7)</f>
+        <v>7</v>
+      </c>
+      <c r="F7" s="19" t="str">
+        <f t="shared" ref="F7:F10" si="1">TEXT(C7,"mmmm")</f>
+        <v>July</v>
+      </c>
+      <c r="G7" s="19" t="str">
+        <f t="shared" ref="G7:G10" si="2">TEXT(C7,"dddd")</f>
+        <v>Friday</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" s="2" t="s">
         <v>127</v>
       </c>
@@ -2856,8 +2942,24 @@
       <c r="C8" s="7">
         <v>46231</v>
       </c>
-    </row>
-    <row r="9" spans="1:3">
+      <c r="D8" s="19">
+        <f>DATEDIF('Exercise-2'!B8,'Exercise-2'!C8,"YD")</f>
+        <v>10</v>
+      </c>
+      <c r="E8" s="19">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="F8" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>July</v>
+      </c>
+      <c r="G8" s="19" t="str">
+        <f t="shared" si="2"/>
+        <v>Tuesday</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
       <c r="A9" s="2" t="s">
         <v>128</v>
       </c>
@@ -2867,8 +2969,24 @@
       <c r="C9" s="7">
         <v>46228</v>
       </c>
-    </row>
-    <row r="10" spans="1:3">
+      <c r="D9" s="19">
+        <f>DATEDIF('Exercise-2'!B9,'Exercise-2'!C9,"YD")</f>
+        <v>5</v>
+      </c>
+      <c r="E9" s="19">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="F9" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>July</v>
+      </c>
+      <c r="G9" s="19" t="str">
+        <f t="shared" si="2"/>
+        <v>Saturday</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" s="2" t="s">
         <v>129</v>
       </c>
@@ -2878,26 +2996,42 @@
       <c r="C10" s="7">
         <v>46232</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="17.5">
+      <c r="D10" s="19">
+        <f>DATEDIF('Exercise-2'!B10,'Exercise-2'!C10,"YD")</f>
+        <v>7</v>
+      </c>
+      <c r="E10" s="19">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="F10" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>July</v>
+      </c>
+      <c r="G10" s="19" t="str">
+        <f t="shared" si="2"/>
+        <v>Wednesday</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="17.5">
       <c r="A12" s="14" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:7">
       <c r="A13" s="15"/>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:7">
       <c r="A14" s="15" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:7">
       <c r="A15" s="15" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:7">
       <c r="A16" s="15" t="s">
         <v>132</v>
       </c>
@@ -2932,90 +3066,191 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{463BC578-FC8A-4D71-8F72-C14B9A00D085}">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.6328125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="31">
+    <row r="1" spans="1:7" ht="31">
       <c r="A1" s="13" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="23.5">
+    <row r="3" spans="1:7" ht="23.5">
       <c r="A3" s="12" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:7" ht="43.5">
       <c r="A5" s="3" t="s">
         <v>135</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="6" spans="1:2">
+      <c r="C5" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="28" t="s">
+        <v>226</v>
+      </c>
+      <c r="E5" s="28" t="s">
+        <v>227</v>
+      </c>
+      <c r="F5" s="28" t="s">
+        <v>228</v>
+      </c>
+      <c r="G5" s="28" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" s="2" t="s">
         <v>137</v>
       </c>
       <c r="B6" s="7">
         <v>38064</v>
       </c>
-    </row>
-    <row r="7" spans="1:2">
+      <c r="C6">
+        <f ca="1">DATEDIF(B6,TODAY(),"Y")</f>
+        <v>22</v>
+      </c>
+      <c r="D6" s="19" t="str">
+        <f>TEXT(B6,"mmmm")</f>
+        <v>March</v>
+      </c>
+      <c r="E6" s="19" t="str">
+        <f>TEXT(B6,"dddd")</f>
+        <v>Thursday</v>
+      </c>
+      <c r="F6" s="19">
+        <f>DAY(B6)</f>
+        <v>18</v>
+      </c>
+      <c r="G6" s="19"/>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B7" s="7">
         <v>38362</v>
       </c>
-    </row>
-    <row r="8" spans="1:2">
+      <c r="C7">
+        <f t="shared" ref="C7:C10" ca="1" si="0">DATEDIF(B7,TODAY(),"Y")</f>
+        <v>21</v>
+      </c>
+      <c r="D7" s="19" t="str">
+        <f t="shared" ref="D7:D10" si="1">TEXT(B7,"mmmm")</f>
+        <v>January</v>
+      </c>
+      <c r="E7" s="19" t="str">
+        <f t="shared" ref="E7:E10" si="2">TEXT(B7,"dddd")</f>
+        <v>Monday</v>
+      </c>
+      <c r="F7" s="19">
+        <f t="shared" ref="F7:F10" si="3">DAY(B7)</f>
+        <v>10</v>
+      </c>
+      <c r="G7" s="19"/>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B8" s="7">
         <v>37947</v>
       </c>
-    </row>
-    <row r="9" spans="1:2">
+      <c r="C8">
+        <f t="shared" ca="1" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="D8" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>November</v>
+      </c>
+      <c r="E8" s="19" t="str">
+        <f t="shared" si="2"/>
+        <v>Saturday</v>
+      </c>
+      <c r="F8" s="19">
+        <f t="shared" si="3"/>
+        <v>22</v>
+      </c>
+      <c r="G8" s="19"/>
+    </row>
+    <row r="9" spans="1:7">
       <c r="A9" s="2" t="s">
         <v>40</v>
       </c>
       <c r="B9" s="7">
         <v>38183</v>
       </c>
-    </row>
-    <row r="10" spans="1:2">
+      <c r="C9">
+        <f t="shared" ca="1" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="D9" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>July</v>
+      </c>
+      <c r="E9" s="19" t="str">
+        <f t="shared" si="2"/>
+        <v>Thursday</v>
+      </c>
+      <c r="F9" s="19">
+        <f t="shared" si="3"/>
+        <v>15</v>
+      </c>
+      <c r="G9" s="19"/>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B10" s="7">
         <v>38845</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" ht="17.5">
+      <c r="C10">
+        <f t="shared" ca="1" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="D10" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>May</v>
+      </c>
+      <c r="E10" s="19" t="str">
+        <f t="shared" si="2"/>
+        <v>Monday</v>
+      </c>
+      <c r="F10" s="19">
+        <f t="shared" si="3"/>
+        <v>8</v>
+      </c>
+      <c r="G10" s="19"/>
+    </row>
+    <row r="12" spans="1:7" ht="17.5">
       <c r="A12" s="14" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:7">
       <c r="A13" s="15"/>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:7">
       <c r="A14" s="15" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:7">
       <c r="A15" s="15" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:7">
       <c r="A16" s="15" t="s">
         <v>140</v>
       </c>

</xml_diff>